<commit_message>
fix(mapeo): hace determinista el generador del mapeo de secciones
El .xlsx cambiaba entre corridas sin que cambiara ningun dato: la tabla de
familias de seccion se construia iterando un set, cuyo orden depende del hash
de Python. Dos familias con el mismo conteo -Introduccion y Metodologia, ambas
21/21- se intercambiaban de fila segun PYTHONHASHSEED.

No afectaba a ninguna cifra, pero rompia la reproducibilidad que este proyecto
exige: dos personas ejecutando el mismo script obtenian archivos distintos.

Corregido: se ordena el set antes de iterarlo y se anaden desempates explicitos
por nombre en las dos tablas de frecuencia que ordenaban solo por conteo.

Verificado con PYTHONHASHSEED 0, 1 y 2: las tres corridas producen el mismo
sha256 sobre el contenido de las celdas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118CSEqQvxD2LbN5hkqoZC6
</commit_message>
<xml_diff>
--- a/docs/entregables/10-mapeo-secciones-articulo/Mapeo-estructura-articulo.xlsx
+++ b/docs/entregables/10-mapeo-secciones-articulo/Mapeo-estructura-articulo.xlsx
@@ -3586,7 +3586,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>proposed methodology</t>
+          <t>background</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
@@ -3597,14 +3597,14 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Metodología / Modelo propuesto</t>
+          <t>Marco teórico previo</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>related works</t>
+          <t>discussion</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3615,14 +3615,14 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Estado del arte</t>
+          <t>Discusión</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>discussion</t>
+          <t>method</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
@@ -3633,14 +3633,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Discusión</t>
+          <t>Metodología / Modelo propuesto</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>background</t>
+          <t>proposed methodology</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3651,14 +3651,14 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Marco teórico previo</t>
+          <t>Metodología / Modelo propuesto</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>method</t>
+          <t>related works</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
@@ -3669,14 +3669,14 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Metodología / Modelo propuesto</t>
+          <t>Estado del arte</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>literature survey</t>
+          <t>literature review</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3694,7 +3694,7 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>literature review</t>
+          <t>literature survey</t>
         </is>
       </c>
       <c r="B77" s="2" t="n">
@@ -3712,7 +3712,7 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>result and discussion</t>
+          <t>proposed model</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -3723,14 +3723,14 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Resultados y discusión (fusionados)</t>
+          <t>Metodología / Modelo propuesto</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>results</t>
+          <t>result and discussion</t>
         </is>
       </c>
       <c r="B79" s="2" t="n">
@@ -3741,14 +3741,14 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Resultados</t>
+          <t>Resultados y discusión (fusionados)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>proposed model</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Metodología / Modelo propuesto</t>
+          <t>Resultados</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3790,7 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Introducción</t>
+          <t>Conclusión</t>
         </is>
       </c>
       <c r="B83" s="2" t="n">
@@ -3804,7 +3804,7 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Metodología / Modelo propuesto</t>
+          <t>Introducción</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -3818,7 +3818,7 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Conclusión</t>
+          <t>Metodología / Modelo propuesto</t>
         </is>
       </c>
       <c r="B85" s="2" t="n">

</xml_diff>

<commit_message>
fix(mapeo): la negrita del Excel se veia como asteriscos literales
45 celdas del entregable mostraban '**texto**' en vez de texto en negrita.
openpyxl no interpreta Markdown: los marcadores que uso el generador se
escribieron tal cual y el lector los veia como asteriscos sueltos.

Corregido con texto enriquecido real (CellRichText + InlineFont): los tramos
entre ** pasan a negrita de Excel y los marcadores desaparecen. Verificado:
0 celdas con asteriscos, 45 con negrita real, y el resultado sigue siendo
identico entre semillas de hash.

Los otros dos .xlsx y los tres .docx no tenian el defecto: sus generadores ya
convertian los marcadores.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118CSEqQvxD2LbN5hkqoZC6
</commit_message>
<xml_diff>
--- a/docs/entregables/10-mapeo-secciones-articulo/Mapeo-estructura-articulo.xlsx
+++ b/docs/entregables/10-mapeo-secciones-articulo/Mapeo-estructura-articulo.xlsx
@@ -703,7 +703,24 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>**21**, por encima del mínimo de 12: **7 semilla de IJIES** (la Opción 1) y 14 de otras revistas — 4 de ISI, 5 de BEEI y 5 de IJSSE</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>21</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, por encima del mínimo de 12: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>7 semilla de IJIES</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (la Opción 1) y 14 de otras revistas — 4 de ISI, 5 de BEEI y 5 de IJSSE</t>
+          </r>
         </is>
       </c>
     </row>
@@ -727,7 +744,18 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Se descargó el PDF completo de cada artículo desde su DOI y se transcribieron los encabezados **tal cual están impresos**, sin normalizar ni traducir. Las erratas del original se conservan y se señalan entre corchetes</t>
+          <r>
+            <t xml:space="preserve">Se descargó el PDF completo de cada artículo desde su DOI y se transcribieron los encabezados </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>tal cual están impresos</t>
+          </r>
+          <r>
+            <t>, sin normalizar ni traducir. Las erratas del original se conservan y se señalan entre corchetes</t>
+          </r>
         </is>
       </c>
     </row>
@@ -3991,7 +4019,15 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>**59 nombres distintos** para 121 secciones de cuerpo</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>59 nombres distintos</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> para 121 secciones de cuerpo</t>
+          </r>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -4008,7 +4044,18 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Solo **2 de 21**: «Introduction» (100 %) y la familia «Conclusión» (100 %)</t>
+          <r>
+            <t xml:space="preserve">Solo </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>2 de 21</t>
+          </r>
+          <r>
+            <t>: «Introduction» (100 %) y la familia «Conclusión» (100 %)</t>
+          </r>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -4025,7 +4072,15 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>**5 nombres** para la misma función: Related work · Related works · Literature review · Literature survey · Materials</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>5 nombres</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> para la misma función: Related work · Related works · Literature review · Literature survey · Materials</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -4042,7 +4097,15 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>**16 nombres distintos**, desde «Methodology» hasta «Hybrid intrusion detection system for 6G»</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>16 nombres distintos</t>
+          </r>
+          <r>
+            <t>, desde «Methodology» hasta «Hybrid intrusion detection system for 6G»</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -4059,7 +4122,18 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Entre **4 y 7** · mediana 5 en IJIES, 6 en el resto</t>
+          <r>
+            <t xml:space="preserve">Entre </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>4 y 7</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> · mediana 5 en IJIES, 6 en el resto</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -4093,12 +4167,31 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>En IJIES: **Conflicts of Interest 7/7 y Author Contributions 7/7**; Acknowledgments 3/7</t>
+          <r>
+            <t xml:space="preserve">En IJIES: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Conflicts of Interest 7/7 y Author Contributions 7/7</t>
+          </r>
+          <r>
+            <t>; Acknowledgments 3/7</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>**Aquí sí hay rigidez**, y es la parte que suele olvidarse</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Aquí sí hay rigidez</t>
+          </r>
+          <r>
+            <t>, y es la parte que suele olvidarse</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4110,7 +4203,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>**No nombra ni una sola sección del cuerpo**</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>No nombra ni una sola sección del cuerpo</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -4209,7 +4307,15 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>**NO.** La guía no nombra ni una sola sección del cuerpo del artículo.</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>NO.</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> La guía no nombra ni una sola sección del cuerpo del artículo.</t>
+          </r>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -4226,12 +4332,34 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>«**Standard number of pages is 8. (The papers must be 8 pages or more.)**»</t>
+          <r>
+            <t>«</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Standard number of pages is 8. (The papers must be 8 pages or more.)</t>
+          </r>
+          <r>
+            <t>»</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Es un **mínimo de 8**, no un máximo. El artículo no puede ser corto.</t>
+          <r>
+            <t xml:space="preserve">Es un </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>mínimo de 8</t>
+          </r>
+          <r>
+            <t>, no un máximo. El artículo no puede ser corto.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4243,12 +4371,52 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>«Extra page charge **USD 50 per extra page** will be requested if the paper length **exceeds 10 pages**.»</t>
+          <r>
+            <t xml:space="preserve">«Extra page charge </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>USD 50 per extra page</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> will be requested if the paper length </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>exceeds 10 pages</t>
+          </r>
+          <r>
+            <t>.»</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>La banda sin sobrecosto es **8 a 10 páginas**. Los 7 semilla miden 10, 11, 12, 13, 14, 16 y 17: **cinco de siete pagaron extra.** Apuntar a 10.</t>
+          <r>
+            <t xml:space="preserve">La banda sin sobrecosto es </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>8 a 10 páginas</t>
+          </r>
+          <r>
+            <t xml:space="preserve">. Los 7 semilla miden 10, 11, 12, 13, 14, 16 y 17: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>cinco de siete pagaron extra.</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Apuntar a 10.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4260,7 +4428,18 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>`IJIES_Format.docx` obligatoria · «extra fee **USD 100** if authors do not use the IJIES_Format.docx»</t>
+          <r>
+            <t xml:space="preserve">`IJIES_Format.docx` obligatoria · «extra fee </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>USD 100</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> if authors do not use the IJIES_Format.docx»</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -4277,7 +4456,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>«The review article (**Survey research**) **is not acceptable** for publication.»</t>
+          <r>
+            <t>«The review article (</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Survey research</t>
+          </r>
+          <r>
+            <t xml:space="preserve">) </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>is not acceptable</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> for publication.»</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4294,12 +4493,43 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dos rondas (1st y 2nd review), «**about 2 weeks**» cada una; dos revisores; notificación en 2 semanas. Decisiones **A / B / C / D**.</t>
+          <r>
+            <t>Dos rondas (1st y 2nd review), «</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>about 2 weeks</t>
+          </r>
+          <r>
+            <t xml:space="preserve">» cada una; dos revisores; notificación en 2 semanas. Decisiones </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>A / B / C / D</t>
+          </r>
+          <r>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Coincide con lo medido: mediana de **41 días** a la primera decisión sobre 5 artículos.</t>
+          <r>
+            <t xml:space="preserve">Coincide con lo medido: mediana de </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>41 días</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a la primera decisión sobre 5 artículos.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4311,29 +4541,84 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mensual · «Accepted papers will be published **about 2 months later**»</t>
+          <r>
+            <t xml:space="preserve">Mensual · «Accepted papers will be published </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>about 2 months later</t>
+          </r>
+          <r>
+            <t>»</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Mediana medida de recepción a publicación: **158 días** (≈5 meses).</t>
+          <r>
+            <t xml:space="preserve">Mediana medida de recepción a publicación: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>158 días</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (≈5 meses).</t>
+          </r>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>**Declaración de uso de IA**</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Declaración de uso de IA</t>
+          </r>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Política propia: «**Transparency regarding substantial AI use is required**». Permite corrección de idioma, depuración de código, organización de ideas y preparación de figuras. **Prohíbe** listar la IA como autor y entregar contenido sin verificación humana.</t>
+          <r>
+            <t>Política propia: «</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Transparency regarding substantial AI use is required</t>
+          </r>
+          <r>
+            <t xml:space="preserve">». Permite corrección de idioma, depuración de código, organización de ideas y preparación de figuras. </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Prohíbe</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> listar la IA como autor y entregar contenido sin verificación humana.</t>
+          </r>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>**Obligatorio declararlo**: el proyecto usó asistentes de IA. Va como sección propia al final.</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Obligatorio declararlo</t>
+          </r>
+          <r>
+            <t>: el proyecto usó asistentes de IA. Va como sección propia al final.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4345,12 +4630,34 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>«upon acceptance, the **copyright of the article will be transferred to the publisher**» · formulario *Copyright Transfer* firmado.</t>
+          <r>
+            <t xml:space="preserve">«upon acceptance, the </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>copyright of the article will be transferred to the publisher</t>
+          </r>
+          <r>
+            <t>» · formulario *Copyright Transfer* firmado.</t>
+          </r>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Explica que su acceso abierto sea **bronce sin licencia**: se lee gratis pero el autor cede el copyright.</t>
+          <r>
+            <t xml:space="preserve">Explica que su acceso abierto sea </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>bronce sin licencia</t>
+          </r>
+          <r>
+            <t>: se lee gratis pero el autor cede el copyright.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4362,7 +4669,18 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>«a fine of **USD 5,000** is requested to authors» si se detecta plagio.</t>
+          <r>
+            <t xml:space="preserve">«a fine of </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>USD 5,000</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> is requested to authors» si se detecta plagio.</t>
+          </r>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -4379,7 +4697,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>«Effective **May 19, 2025**, the submission of cover letters has been rendered **unnecessary**»</t>
+          <r>
+            <t xml:space="preserve">«Effective </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>May 19, 2025</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, the submission of cover letters has been rendered </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>unnecessary</t>
+          </r>
+          <r>
+            <t>»</t>
+          </r>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -4396,12 +4734,43 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>«**Paypal (Credit card) is the only payment method**. The bank transfer is **not supported**.»</t>
+          <r>
+            <t>«</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Paypal (Credit card) is the only payment method</t>
+          </r>
+          <r>
+            <t xml:space="preserve">. The bank transfer is </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>not supported</t>
+          </r>
+          <r>
+            <t>.»</t>
+          </r>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Resolver el medio de pago **antes** de enviar.</t>
+          <r>
+            <t xml:space="preserve">Resolver el medio de pago </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>antes</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> de enviar.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4413,7 +4782,18 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>USD 300 hoy · **USD 400 desde el 1 de octubre de 2026** (incluye ya el cargo de formato)</t>
+          <r>
+            <t xml:space="preserve">USD 300 hoy · </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>USD 400 desde el 1 de octubre de 2026</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> (incluye ya el cargo de formato)</t>
+          </r>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -4524,7 +4904,15 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>21/21 — **100 %**</t>
+          <r>
+            <t xml:space="preserve">21/21 — </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>100 %</t>
+          </r>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -4551,7 +4939,18 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>13/21 con ese nombre · **19/21 (90 %)** como familia</t>
+          <r>
+            <t xml:space="preserve">13/21 con ese nombre · </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>19/21 (90 %)</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> como familia</t>
+          </r>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -4578,7 +4977,15 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>**21/21 — 100 %** como familia</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>21/21 — 100 %</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> como familia</t>
+          </r>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -4588,7 +4995,18 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio, dataset multilayer-v2, las 28 variables, ventanas, OCSVM y calibración del umbral. Sección más extensa (hasta 36 párrafos en la muestra). El dataset va **aquí como subsección**, no como sección aparte (así en 3 de 4 revistas).</t>
+          <r>
+            <t xml:space="preserve">Laboratorio, dataset multilayer-v2, las 28 variables, ventanas, OCSVM y calibración del umbral. Sección más extensa (hasta 36 párrafos en la muestra). El dataset va </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>aquí como subsección</t>
+          </r>
+          <r>
+            <t>, no como sección aparte (así en 3 de 4 revistas).</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4605,12 +5023,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>**11/21 fusionados** · 10/21 separados</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>11/21 fusionados</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> · 10/21 separados</t>
+          </r>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Guía: no la nombra · Mapeo: **fusionar es lo más frecuente en IJIES (5/7)**</t>
+          <r>
+            <t xml:space="preserve">Guía: no la nombra · Mapeo: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>fusionar es lo más frecuente en IJIES (5/7)</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -4632,7 +5066,15 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>21/21 — **100 %**</t>
+          <r>
+            <t xml:space="preserve">21/21 — </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>100 %</t>
+          </r>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4642,7 +5084,18 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sin citas: **0 de 21 artículos citan en la conclusión**. Cierre y trabajo futuro.</t>
+          <r>
+            <t xml:space="preserve">Sin citas: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>0 de 21 artículos citan en la conclusión</t>
+          </r>
+          <r>
+            <t>. Cierre y trabajo futuro.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4659,7 +5112,15 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>7/7 en IJIES — **100 %**</t>
+          <r>
+            <t xml:space="preserve">7/7 en IJIES — </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>100 %</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4686,7 +5147,15 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>7/7 en IJIES — **100 %**</t>
+          <r>
+            <t xml:space="preserve">7/7 en IJIES — </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>100 %</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -4718,12 +5187,28 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>**Guía: obligatoria** («transparency regarding substantial AI use is required») · Mapeo: aún no aparece</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>Guía: obligatoria</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> («transparency regarding substantial AI use is required») · Mapeo: aún no aparece</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>**La exige la guía aunque no esté en los artículos de 2024.** Qué asistió la IA y qué verificaron los autores.</t>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>La exige la guía aunque no esté en los artículos de 2024.</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Qué asistió la IA y qué verificaron los autores.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -4767,7 +5252,15 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>21/21 — **100 %**</t>
+          <r>
+            <t xml:space="preserve">21/21 — </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>100 %</t>
+          </r>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -4777,7 +5270,18 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Rango observado en IJIES: **17 a 49**, mediana 39.</t>
+          <r>
+            <t xml:space="preserve">Rango observado en IJIES: </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>17 a 49</t>
+          </r>
+          <r>
+            <t>, mediana 39.</t>
+          </r>
         </is>
       </c>
     </row>

</xml_diff>